<commit_message>
Update Web production backend and socket URLs to deployed Render service
</commit_message>
<xml_diff>
--- a/LifeLinkTesting/reports/excel/LifeLink_Web_500_Test_Report.xlsx
+++ b/LifeLinkTesting/reports/excel/LifeLink_Web_500_Test_Report.xlsx
@@ -73,13 +73,13 @@
     <t>Total Execution Duration</t>
   </si>
   <si>
-    <t>1.250 s</t>
+    <t>1.251 s</t>
   </si>
   <si>
     <t>Production Backend URL</t>
   </si>
   <si>
-    <t>http://localhost:5000/api</t>
+    <t>https://lifelink-backend-avuk.onrender.com/api</t>
   </si>
   <si>
     <t>GitHub Pages URL</t>

</xml_diff>